<commit_message>
Updated quantitative analysis code
</commit_message>
<xml_diff>
--- a/quantitative/analysis/figures/analysis/overall_factor_summary.xlsx
+++ b/quantitative/analysis/figures/analysis/overall_factor_summary.xlsx
@@ -423,37 +423,37 @@
         </is>
       </c>
       <c r="B2">
-        <v>3873</v>
+        <v>7069</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>23</v>
+        <v>133</v>
       </c>
       <c r="E2">
-        <v>4.17</v>
+        <v>4.14</v>
       </c>
       <c r="F2">
-        <v>4.04</v>
+        <v>4</v>
       </c>
       <c r="G2">
-        <v>4.3</v>
+        <v>4.29</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>0.134</v>
       </c>
       <c r="I2">
-        <v>0.227</v>
+        <v>0.212</v>
       </c>
       <c r="J2">
-        <v>0.406</v>
+        <v>0.378</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="L2">
-        <v>0.239</v>
+        <v>0.218</v>
       </c>
     </row>
     <row r="3">
@@ -463,37 +463,37 @@
         </is>
       </c>
       <c r="B3">
-        <v>3872</v>
+        <v>6478</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>23</v>
+        <v>133</v>
       </c>
       <c r="E3">
-        <v>3.65</v>
+        <v>3.68</v>
       </c>
       <c r="F3">
-        <v>3.26</v>
+        <v>3.35</v>
       </c>
       <c r="G3">
-        <v>4.04</v>
+        <v>4.01</v>
       </c>
       <c r="H3">
-        <v>0.439</v>
+        <v>0.29</v>
       </c>
       <c r="I3">
-        <v>0.07099999999999999</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="J3">
-        <v>0.695</v>
+        <v>0.73</v>
       </c>
       <c r="K3">
-        <v>0.283</v>
+        <v>0.09</v>
       </c>
       <c r="L3">
-        <v>0.007</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="4">
@@ -503,37 +503,37 @@
         </is>
       </c>
       <c r="B4">
-        <v>3871</v>
+        <v>6830</v>
       </c>
       <c r="C4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>23</v>
+        <v>133</v>
       </c>
       <c r="E4">
-        <v>3.99</v>
+        <v>3.9</v>
       </c>
       <c r="F4">
-        <v>3.86</v>
+        <v>3.57</v>
       </c>
       <c r="G4">
-        <v>4.12</v>
+        <v>4.24</v>
       </c>
       <c r="H4">
-        <v>0.136</v>
+        <v>0.275</v>
       </c>
       <c r="I4">
-        <v>0.064</v>
+        <v>0.708</v>
       </c>
       <c r="J4">
-        <v>0.492</v>
+        <v>0.449</v>
       </c>
       <c r="K4">
-        <v>0.07000000000000001</v>
+        <v>0.097</v>
       </c>
       <c r="L4">
-        <v>0.015</v>
+        <v>0.643</v>
       </c>
     </row>
   </sheetData>

</xml_diff>